<commit_message>
Restructure Market - Demand-Side Scan section
- Remove Primary Demand Drivers chart entirely (HTML, JS, and its unused
  data template)
- Move Demand Growth by Channel below Penetration by Range & Customer
  Type, as its own full-width panel
- Remove all stat cards, replace with a single New Product Growth card;
  sync data/Market - Demand-Side Scan - Stat Cards.xlsx to match

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Market - Demand-Side Scan - Stat Cards.xlsx
+++ b/data/Market - Demand-Side Scan - Stat Cards.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -451,51 +451,18 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Regional Dairy Category Growth</t>
+          <t>New Product Growth</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>retail volume, YoY</t>
+          <t>revenue from SKUs launched in past 12 mo</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Local/Premium Segment Share</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>% of category retail $</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>School/Institutional Demand</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>contract volume growth</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Direct-to-Consumer Growth</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>farm store &amp; online</t>
-        </is>
-      </c>
-    </row>
+    <row r="3"/>
+    <row r="4"/>
+    <row r="5"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fill in New Product Growth stat card
$2,339,042 total revenue from new SKUs, May 2025-Jun 2026. Dropped the
vs-TTM-Jul-2025 delta line since a YoY comparison doesn't apply to a new
product launch metric. Sync data/Market - Demand-Side Scan - Stat Cards.xlsx.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Market - Demand-Side Scan - Stat Cards.xlsx
+++ b/data/Market - Demand-Side Scan - Stat Cards.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -456,13 +456,13 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>revenue from SKUs launched in past 12 mo</t>
-        </is>
+          <t>total revenue, new SKUs, May 2025-Jun 2026</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>2339042</v>
       </c>
     </row>
-    <row r="3"/>
-    <row r="4"/>
-    <row r="5"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>